<commit_message>
data(catalog): update composition source data for enriched domain model
</commit_message>
<xml_diff>
--- a/app/excel_files/base_composicoes_v2.xlsx
+++ b/app/excel_files/base_composicoes_v2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\sinapi+\app\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C36AE59-5645-4B2D-BA00-9A6B18402600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DDD3D3A-F0FC-43A1-9240-6CCBF1662B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="113">
   <si>
     <t>grupo</t>
   </si>
@@ -372,6 +372,9 @@
   </si>
   <si>
     <t>Composição</t>
+  </si>
+  <si>
+    <t>unidade_composicao_secundaria</t>
   </si>
 </sst>
 </file>
@@ -425,7 +428,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -443,9 +449,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela1" displayName="Tabela1" ref="A1:H153" totalsRowShown="0">
-  <autoFilter ref="A1:H153" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela1" displayName="Tabela1" ref="A1:I153" totalsRowShown="0">
+  <autoFilter ref="A1:I153" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="grupo"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="codigo_composicao"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="descricao_da_composicao"/>
@@ -453,7 +459,8 @@
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="coeficiente"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="codigo_composicao_secundaria"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="descricao_da_composicao_secundaria"/>
-    <tableColumn id="8" xr3:uid="{E8FC14DE-BC4A-4B86-973A-7FB96BB5FE0E}" name="tipo" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{EDFFBBE4-DCE6-4903-BF85-558CADFBD3A9}" name="unidade_composicao_secundaria" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{E8FC14DE-BC4A-4B86-973A-7FB96BB5FE0E}" name="tipo" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -635,7 +642,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H162"/>
+  <dimension ref="A1:I162"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" customWidth="1"/>
@@ -644,12 +651,12 @@
     <col min="4" max="4" width="10.5703125" customWidth="1"/>
     <col min="5" max="5" width="13.5703125" customWidth="1"/>
     <col min="6" max="6" width="38.5703125" customWidth="1"/>
-    <col min="7" max="7" width="87.28515625" customWidth="1"/>
-    <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="16382" max="16384" width="13.42578125" customWidth="1"/>
+    <col min="7" max="8" width="87.28515625" customWidth="1"/>
+    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="16383" max="16384" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -671,11 +678,14 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="I1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -697,11 +707,14 @@
       <c r="G2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="H2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -723,11 +736,14 @@
       <c r="G3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="H3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -749,11 +765,14 @@
       <c r="G4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -775,11 +794,14 @@
       <c r="G5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -801,11 +823,14 @@
       <c r="G6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H6" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
@@ -827,11 +852,14 @@
       <c r="G7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="H7" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -853,11 +881,14 @@
       <c r="G8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H8" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -879,11 +910,14 @@
       <c r="G9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="H9" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H9" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I9" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
@@ -905,11 +939,14 @@
       <c r="G10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H10" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H10" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
@@ -931,11 +968,14 @@
       <c r="G11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H11" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>7</v>
       </c>
@@ -957,11 +997,14 @@
       <c r="G12" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H12" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I12" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>7</v>
       </c>
@@ -983,11 +1026,14 @@
       <c r="G13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H13" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I13" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>7</v>
       </c>
@@ -1009,11 +1055,14 @@
       <c r="G14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H14" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H14" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I14" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>7</v>
       </c>
@@ -1035,11 +1084,14 @@
       <c r="G15" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>7</v>
       </c>
@@ -1061,11 +1113,14 @@
       <c r="G16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H16" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H16" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>7</v>
       </c>
@@ -1087,11 +1142,14 @@
       <c r="G17" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H17" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H17" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I17" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>7</v>
       </c>
@@ -1113,11 +1171,14 @@
       <c r="G18" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H18" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H18" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>7</v>
       </c>
@@ -1139,11 +1200,14 @@
       <c r="G19" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H19" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H19" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>7</v>
       </c>
@@ -1165,11 +1229,14 @@
       <c r="G20" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H20" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I20" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>7</v>
       </c>
@@ -1191,11 +1258,14 @@
       <c r="G21" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H21" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H21" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I21" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>7</v>
       </c>
@@ -1217,11 +1287,14 @@
       <c r="G22" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H22" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H22" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>7</v>
       </c>
@@ -1243,11 +1316,14 @@
       <c r="G23" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H23" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I23" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>7</v>
       </c>
@@ -1269,11 +1345,14 @@
       <c r="G24" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H24" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H24" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I24" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>7</v>
       </c>
@@ -1295,11 +1374,14 @@
       <c r="G25" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H25" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H25" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I25" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>7</v>
       </c>
@@ -1321,11 +1403,14 @@
       <c r="G26" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="H26" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H26" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I26" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>7</v>
       </c>
@@ -1347,11 +1432,14 @@
       <c r="G27" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H27" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H27" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I27" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>7</v>
       </c>
@@ -1373,11 +1461,14 @@
       <c r="G28" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H28" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H28" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I28" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>7</v>
       </c>
@@ -1399,11 +1490,14 @@
       <c r="G29" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H29" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H29" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I29" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>7</v>
       </c>
@@ -1425,11 +1519,14 @@
       <c r="G30" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H30" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H30" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I30" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>7</v>
       </c>
@@ -1451,11 +1548,14 @@
       <c r="G31" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="H31" t="s">
+      <c r="H31" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I31" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>7</v>
       </c>
@@ -1477,11 +1577,14 @@
       <c r="G32" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H32" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H32" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I32" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>7</v>
       </c>
@@ -1503,11 +1606,14 @@
       <c r="G33" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H33" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H33" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I33" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>7</v>
       </c>
@@ -1529,11 +1635,14 @@
       <c r="G34" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="H34" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H34" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I34" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>7</v>
       </c>
@@ -1555,11 +1664,14 @@
       <c r="G35" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H35" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H35" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I35" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>7</v>
       </c>
@@ -1581,11 +1693,14 @@
       <c r="G36" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H36" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H36" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I36" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>7</v>
       </c>
@@ -1607,11 +1722,14 @@
       <c r="G37" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H37" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H37" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I37" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>7</v>
       </c>
@@ -1633,11 +1751,14 @@
       <c r="G38" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H38" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H38" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I38" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>7</v>
       </c>
@@ -1659,11 +1780,14 @@
       <c r="G39" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H39" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H39" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I39" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>7</v>
       </c>
@@ -1685,11 +1809,14 @@
       <c r="G40" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H40" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H40" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I40" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>7</v>
       </c>
@@ -1711,11 +1838,14 @@
       <c r="G41" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="H41" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H41" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I41" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>7</v>
       </c>
@@ -1737,11 +1867,14 @@
       <c r="G42" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H42" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H42" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I42" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>7</v>
       </c>
@@ -1763,11 +1896,14 @@
       <c r="G43" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="H43" t="s">
+      <c r="H43" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I43" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>7</v>
       </c>
@@ -1789,11 +1925,14 @@
       <c r="G44" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H44" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H44" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I44" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>7</v>
       </c>
@@ -1815,11 +1954,14 @@
       <c r="G45" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H45" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H45" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I45" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>7</v>
       </c>
@@ -1841,11 +1983,14 @@
       <c r="G46" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H46" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H46" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I46" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>7</v>
       </c>
@@ -1867,11 +2012,14 @@
       <c r="G47" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H47" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H47" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I47" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>7</v>
       </c>
@@ -1893,11 +2041,14 @@
       <c r="G48" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H48" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H48" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I48" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>7</v>
       </c>
@@ -1919,11 +2070,14 @@
       <c r="G49" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H49" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H49" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I49" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>7</v>
       </c>
@@ -1945,11 +2099,14 @@
       <c r="G50" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="H50" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H50" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I50" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>7</v>
       </c>
@@ -1971,11 +2128,14 @@
       <c r="G51" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H51" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H51" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I51" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>7</v>
       </c>
@@ -1997,11 +2157,14 @@
       <c r="G52" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="H52" t="s">
+      <c r="H52" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I52" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>7</v>
       </c>
@@ -2023,11 +2186,14 @@
       <c r="G53" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H53" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H53" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I53" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>7</v>
       </c>
@@ -2049,11 +2215,14 @@
       <c r="G54" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H54" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H54" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I54" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>7</v>
       </c>
@@ -2075,11 +2244,14 @@
       <c r="G55" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H55" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H55" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I55" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>7</v>
       </c>
@@ -2101,11 +2273,14 @@
       <c r="G56" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H56" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H56" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I56" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>7</v>
       </c>
@@ -2127,11 +2302,14 @@
       <c r="G57" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H57" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H57" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I57" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>7</v>
       </c>
@@ -2153,11 +2331,14 @@
       <c r="G58" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H58" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H58" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I58" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>7</v>
       </c>
@@ -2179,11 +2360,14 @@
       <c r="G59" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="H59" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H59" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I59" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>7</v>
       </c>
@@ -2205,11 +2389,14 @@
       <c r="G60" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H60" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H60" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I60" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>7</v>
       </c>
@@ -2231,11 +2418,14 @@
       <c r="G61" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="H61" t="s">
+      <c r="H61" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I61" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>7</v>
       </c>
@@ -2257,11 +2447,14 @@
       <c r="G62" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H62" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H62" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I62" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>7</v>
       </c>
@@ -2283,11 +2476,14 @@
       <c r="G63" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H63" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H63" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I63" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>7</v>
       </c>
@@ -2309,11 +2505,14 @@
       <c r="G64" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H64" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H64" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I64" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>7</v>
       </c>
@@ -2335,11 +2534,14 @@
       <c r="G65" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H65" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H65" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I65" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>7</v>
       </c>
@@ -2361,11 +2563,14 @@
       <c r="G66" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H66" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H66" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I66" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>7</v>
       </c>
@@ -2387,11 +2592,14 @@
       <c r="G67" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H67" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H67" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I67" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>7</v>
       </c>
@@ -2413,11 +2621,14 @@
       <c r="G68" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="H68" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H68" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I68" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>7</v>
       </c>
@@ -2439,11 +2650,14 @@
       <c r="G69" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H69" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H69" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I69" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>7</v>
       </c>
@@ -2465,11 +2679,14 @@
       <c r="G70" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="H70" t="s">
+      <c r="H70" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I70" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>7</v>
       </c>
@@ -2491,11 +2708,14 @@
       <c r="G71" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H71" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H71" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I71" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>63</v>
       </c>
@@ -2517,11 +2737,14 @@
       <c r="G72" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H72" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H72" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I72" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>63</v>
       </c>
@@ -2543,11 +2766,14 @@
       <c r="G73" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H73" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="74" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H73" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I73" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>63</v>
       </c>
@@ -2569,11 +2795,14 @@
       <c r="G74" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H74" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="75" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H74" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I74" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>63</v>
       </c>
@@ -2595,11 +2824,14 @@
       <c r="G75" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="H75" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="76" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H75" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I75" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>63</v>
       </c>
@@ -2621,11 +2853,14 @@
       <c r="G76" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H76" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="77" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H76" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I76" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>63</v>
       </c>
@@ -2647,11 +2882,14 @@
       <c r="G77" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="H77" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="78" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H77" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I77" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>63</v>
       </c>
@@ -2673,11 +2911,14 @@
       <c r="G78" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H78" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H78" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I78" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>63</v>
       </c>
@@ -2699,11 +2940,14 @@
       <c r="G79" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H79" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="80" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H79" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I79" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>63</v>
       </c>
@@ -2725,11 +2969,14 @@
       <c r="G80" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H80" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="81" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H80" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I80" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>63</v>
       </c>
@@ -2751,11 +2998,14 @@
       <c r="G81" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H81" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="82" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H81" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I81" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>63</v>
       </c>
@@ -2777,11 +3027,14 @@
       <c r="G82" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="H82" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="83" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H82" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I82" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>63</v>
       </c>
@@ -2803,11 +3056,14 @@
       <c r="G83" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H83" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="84" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H83" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I83" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>63</v>
       </c>
@@ -2829,11 +3085,14 @@
       <c r="G84" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H84" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H84" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I84" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>63</v>
       </c>
@@ -2855,11 +3114,14 @@
       <c r="G85" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="H85" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="86" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H85" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I85" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>63</v>
       </c>
@@ -2881,11 +3143,14 @@
       <c r="G86" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="H86" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="87" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H86" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I86" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>63</v>
       </c>
@@ -2907,11 +3172,14 @@
       <c r="G87" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="H87" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="88" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H87" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I87" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>63</v>
       </c>
@@ -2933,11 +3201,14 @@
       <c r="G88" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H88" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="89" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H88" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I88" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>63</v>
       </c>
@@ -2959,11 +3230,14 @@
       <c r="G89" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="H89" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="90" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H89" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I89" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>63</v>
       </c>
@@ -2985,11 +3259,14 @@
       <c r="G90" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="H90" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="91" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H90" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I90" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>63</v>
       </c>
@@ -3011,11 +3288,14 @@
       <c r="G91" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="H91" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="92" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H91" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I91" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>63</v>
       </c>
@@ -3037,11 +3317,14 @@
       <c r="G92" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H92" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="93" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H92" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I92" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>63</v>
       </c>
@@ -3063,11 +3346,14 @@
       <c r="G93" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="H93" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="94" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H93" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I93" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>63</v>
       </c>
@@ -3089,11 +3375,14 @@
       <c r="G94" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="H94" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="95" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H94" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I94" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>63</v>
       </c>
@@ -3115,11 +3404,14 @@
       <c r="G95" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="H95" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="96" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H95" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I95" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>63</v>
       </c>
@@ -3141,11 +3433,14 @@
       <c r="G96" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="H96" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="97" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H96" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I96" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>63</v>
       </c>
@@ -3167,11 +3462,14 @@
       <c r="G97" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H97" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="98" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H97" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I97" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>63</v>
       </c>
@@ -3193,11 +3491,14 @@
       <c r="G98" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H98" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="99" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H98" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I98" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>63</v>
       </c>
@@ -3219,11 +3520,14 @@
       <c r="G99" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H99" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="100" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H99" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I99" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>63</v>
       </c>
@@ -3245,11 +3549,14 @@
       <c r="G100" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="H100" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="101" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H100" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I100" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>63</v>
       </c>
@@ -3271,11 +3578,14 @@
       <c r="G101" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H101" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="102" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H101" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I101" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>63</v>
       </c>
@@ -3297,11 +3607,14 @@
       <c r="G102" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="H102" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="103" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H102" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I102" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>63</v>
       </c>
@@ -3323,11 +3636,14 @@
       <c r="G103" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H103" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="104" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H103" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I103" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>63</v>
       </c>
@@ -3349,11 +3665,14 @@
       <c r="G104" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="H104" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="105" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H104" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I104" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>63</v>
       </c>
@@ -3375,11 +3694,14 @@
       <c r="G105" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="H105" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="106" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H105" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I105" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>63</v>
       </c>
@@ -3401,11 +3723,14 @@
       <c r="G106" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="H106" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="107" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H106" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I106" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>63</v>
       </c>
@@ -3427,11 +3752,14 @@
       <c r="G107" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H107" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="108" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H107" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I107" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>63</v>
       </c>
@@ -3453,11 +3781,14 @@
       <c r="G108" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H108" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="109" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H108" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I108" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>63</v>
       </c>
@@ -3479,11 +3810,14 @@
       <c r="G109" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H109" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="110" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H109" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I109" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>63</v>
       </c>
@@ -3505,11 +3839,14 @@
       <c r="G110" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="H110" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="111" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H110" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I110" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>63</v>
       </c>
@@ -3531,11 +3868,14 @@
       <c r="G111" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H111" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="112" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H111" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I111" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>63</v>
       </c>
@@ -3557,11 +3897,14 @@
       <c r="G112" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="H112" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="113" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H112" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I112" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>63</v>
       </c>
@@ -3583,11 +3926,14 @@
       <c r="G113" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H113" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="114" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H113" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I113" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>63</v>
       </c>
@@ -3609,11 +3955,14 @@
       <c r="G114" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H114" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="115" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H114" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I114" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>63</v>
       </c>
@@ -3635,11 +3984,14 @@
       <c r="G115" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H115" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="116" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H115" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I115" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>63</v>
       </c>
@@ -3661,11 +4013,14 @@
       <c r="G116" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H116" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="117" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H116" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I116" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>63</v>
       </c>
@@ -3687,11 +4042,14 @@
       <c r="G117" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H117" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="118" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H117" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I117" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>63</v>
       </c>
@@ -3713,11 +4071,14 @@
       <c r="G118" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H118" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="119" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H118" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I118" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>63</v>
       </c>
@@ -3739,11 +4100,14 @@
       <c r="G119" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H119" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="120" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H119" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I119" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>63</v>
       </c>
@@ -3765,11 +4129,14 @@
       <c r="G120" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H120" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="121" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H120" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I120" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>63</v>
       </c>
@@ -3791,11 +4158,14 @@
       <c r="G121" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H121" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="122" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H121" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I121" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>63</v>
       </c>
@@ -3817,11 +4187,14 @@
       <c r="G122" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H122" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="123" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H122" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I122" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>63</v>
       </c>
@@ -3843,11 +4216,14 @@
       <c r="G123" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="H123" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="124" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H123" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I123" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>63</v>
       </c>
@@ -3869,11 +4245,14 @@
       <c r="G124" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H124" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="125" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H124" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I124" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>63</v>
       </c>
@@ -3895,11 +4274,14 @@
       <c r="G125" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H125" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="126" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H125" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I125" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>63</v>
       </c>
@@ -3921,11 +4303,14 @@
       <c r="G126" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H126" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="127" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H126" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I126" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>63</v>
       </c>
@@ -3947,11 +4332,14 @@
       <c r="G127" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H127" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="128" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H127" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I127" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>63</v>
       </c>
@@ -3973,11 +4361,14 @@
       <c r="G128" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H128" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="129" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H128" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I128" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>63</v>
       </c>
@@ -3999,11 +4390,14 @@
       <c r="G129" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H129" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="130" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H129" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I129" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>63</v>
       </c>
@@ -4025,11 +4419,14 @@
       <c r="G130" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="H130" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="131" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H130" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I130" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>63</v>
       </c>
@@ -4051,11 +4448,14 @@
       <c r="G131" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H131" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="132" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H131" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I131" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>63</v>
       </c>
@@ -4077,11 +4477,14 @@
       <c r="G132" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H132" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="133" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H132" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I132" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>63</v>
       </c>
@@ -4103,11 +4506,14 @@
       <c r="G133" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H133" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="134" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H133" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I133" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>63</v>
       </c>
@@ -4129,11 +4535,14 @@
       <c r="G134" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H134" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="135" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H134" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I134" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
         <v>63</v>
       </c>
@@ -4155,11 +4564,14 @@
       <c r="G135" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H135" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="136" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H135" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I135" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>63</v>
       </c>
@@ -4181,11 +4593,14 @@
       <c r="G136" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H136" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="137" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H136" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I136" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
         <v>63</v>
       </c>
@@ -4207,11 +4622,14 @@
       <c r="G137" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="H137" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="138" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H137" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I137" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>63</v>
       </c>
@@ -4233,11 +4651,14 @@
       <c r="G138" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H138" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="139" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H138" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I138" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>63</v>
       </c>
@@ -4259,11 +4680,14 @@
       <c r="G139" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H139" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="140" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H139" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I139" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
         <v>63</v>
       </c>
@@ -4285,11 +4709,14 @@
       <c r="G140" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H140" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="141" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H140" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I140" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>63</v>
       </c>
@@ -4311,11 +4738,14 @@
       <c r="G141" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H141" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="142" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H141" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I141" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>63</v>
       </c>
@@ -4337,11 +4767,14 @@
       <c r="G142" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H142" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="143" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H142" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I142" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
         <v>63</v>
       </c>
@@ -4363,11 +4796,14 @@
       <c r="G143" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H143" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="144" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H143" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I143" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>63</v>
       </c>
@@ -4389,11 +4825,14 @@
       <c r="G144" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="H144" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="145" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H144" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I144" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>63</v>
       </c>
@@ -4415,11 +4854,14 @@
       <c r="G145" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H145" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="146" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H145" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I145" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>63</v>
       </c>
@@ -4441,11 +4883,14 @@
       <c r="G146" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H146" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="147" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H146" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I146" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
         <v>63</v>
       </c>
@@ -4467,11 +4912,14 @@
       <c r="G147" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H147" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="148" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H147" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I147" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>63</v>
       </c>
@@ -4493,11 +4941,14 @@
       <c r="G148" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H148" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="149" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H148" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I148" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>63</v>
       </c>
@@ -4519,11 +4970,14 @@
       <c r="G149" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H149" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="150" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="H149" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I149" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>63</v>
       </c>
@@ -4545,11 +4999,14 @@
       <c r="G150" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H150" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="151" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H150" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I150" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>63</v>
       </c>
@@ -4571,11 +5028,14 @@
       <c r="G151" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="H151" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="152" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="H151" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I151" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>63</v>
       </c>
@@ -4597,11 +5057,14 @@
       <c r="G152" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H152" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="153" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H152" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I152" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>63</v>
       </c>
@@ -4623,11 +5086,14 @@
       <c r="G153" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H153" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="154" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H153" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I153" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A154" s="2"/>
       <c r="B154" s="2"/>
       <c r="C154" s="3"/>
@@ -4635,41 +5101,49 @@
       <c r="E154" s="4"/>
       <c r="F154" s="2"/>
       <c r="G154" s="3"/>
-    </row>
-    <row r="155" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H154" s="3"/>
+    </row>
+    <row r="155" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="C155" s="3"/>
       <c r="F155" s="2"/>
       <c r="G155" s="3"/>
-    </row>
-    <row r="156" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H155" s="3"/>
+    </row>
+    <row r="156" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="C156" s="3"/>
       <c r="F156" s="2"/>
       <c r="G156" s="3"/>
-    </row>
-    <row r="157" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H156" s="3"/>
+    </row>
+    <row r="157" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="C157" s="3"/>
       <c r="F157" s="2"/>
       <c r="G157" s="3"/>
-    </row>
-    <row r="158" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H157" s="3"/>
+    </row>
+    <row r="158" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="C158" s="3"/>
       <c r="F158" s="2"/>
       <c r="G158" s="3"/>
-    </row>
-    <row r="159" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H158" s="3"/>
+    </row>
+    <row r="159" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="C159" s="3"/>
       <c r="F159" s="2"/>
       <c r="G159" s="3"/>
-    </row>
-    <row r="160" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H159" s="3"/>
+    </row>
+    <row r="160" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="C160" s="3"/>
       <c r="F160" s="2"/>
       <c r="G160" s="3"/>
-    </row>
-    <row r="161" spans="6:7" ht="15" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="6:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="H160" s="3"/>
+    </row>
+    <row r="161" spans="6:8" ht="15" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="6:8" ht="15" x14ac:dyDescent="0.25">
       <c r="F162" s="2"/>
       <c r="G162" s="3"/>
+      <c r="H162" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>